<commit_message>
[进度] 10-15 重新生成 (V0 94.6%)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-15.xlsx
+++ b/docs/progress/显性目的进度_2026-10-15.xlsx
@@ -8261,7 +8261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J107"/>
+  <dimension ref="A1:J109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9479,51 +9479,51 @@
     </row>
     <row r="54">
       <c r="A54" s="18" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B54" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46310</v>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>QoS</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>上行出口全量复验 45/0, 合主线</t>
+          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 fdb4de6</t>
+          <t>~/qos_runs</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="18" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+        <v>46310</v>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D16b</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
+          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>scratchpad/v_pls4_board.log</t>
+          <t>dr1v90 task/d16b-tile 7936b7e</t>
         </is>
       </c>
     </row>
@@ -9531,24 +9531,24 @@
       <c r="A56" s="18" t="n">
         <v>46309</v>
       </c>
-      <c r="B56" s="16" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B56" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
+          <t>上行出口全量复验 45/0, 合主线</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>dr1v90 fdb4de6</t>
         </is>
       </c>
     </row>
@@ -9556,24 +9556,24 @@
       <c r="A57" s="18" t="n">
         <v>46309</v>
       </c>
-      <c r="B57" s="16" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
+          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>scratchpad/v_pls4_board.log</t>
         </is>
       </c>
     </row>
@@ -9581,24 +9581,24 @@
       <c r="A58" s="18" t="n">
         <v>46309</v>
       </c>
-      <c r="B58" s="19" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
+          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>project_short_term_delivery_1013</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -9613,17 +9613,17 @@
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
+          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 debd3cd</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -9631,24 +9631,24 @@
       <c r="A60" s="18" t="n">
         <v>46309</v>
       </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B60" s="19" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
+          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>scratchpad v_pls6_board.log</t>
+          <t>project_short_term_delivery_1013</t>
         </is>
       </c>
     </row>
@@ -9656,9 +9656,9 @@
       <c r="A61" s="18" t="n">
         <v>46309</v>
       </c>
-      <c r="B61" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
@@ -9668,12 +9668,12 @@
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
+          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>dr1v90 task/pls-2047 debd3cd</t>
         </is>
       </c>
     </row>
@@ -9681,24 +9681,24 @@
       <c r="A62" s="18" t="n">
         <v>46309</v>
       </c>
-      <c r="B62" s="16" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
+          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16-ddr 539d303</t>
+          <t>scratchpad v_pls6_board.log</t>
         </is>
       </c>
     </row>
@@ -9706,24 +9706,24 @@
       <c r="A63" s="18" t="n">
         <v>46309</v>
       </c>
-      <c r="B63" s="19" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
+          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>feedback_save_weekly_quota</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -9731,24 +9731,24 @@
       <c r="A64" s="18" t="n">
         <v>46309</v>
       </c>
-      <c r="B64" s="20" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B64" s="16" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
+          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>dr1v90 task/d16-ddr 539d303</t>
         </is>
       </c>
     </row>
@@ -9756,24 +9756,24 @@
       <c r="A65" s="18" t="n">
         <v>46309</v>
       </c>
-      <c r="B65" s="14" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B65" s="19" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
+          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 2364e5c</t>
+          <t>feedback_save_weekly_quota</t>
         </is>
       </c>
     </row>
@@ -9788,17 +9788,17 @@
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
+          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>用户在场实转</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -9806,24 +9806,24 @@
       <c r="A67" s="18" t="n">
         <v>46309</v>
       </c>
-      <c r="B67" s="19" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B67" s="14" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
+          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 2364e5c</t>
         </is>
       </c>
     </row>
@@ -9831,24 +9831,24 @@
       <c r="A68" s="18" t="n">
         <v>46309</v>
       </c>
-      <c r="B68" s="14" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B68" s="20" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
+          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>用户在场实转</t>
         </is>
       </c>
     </row>
@@ -9863,12 +9863,12 @@
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
+          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
@@ -9888,17 +9888,17 @@
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
+          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 dee9be6</t>
+          <t>dr1v90 task/d18-pl-default d35c6d4</t>
         </is>
       </c>
     </row>
@@ -9906,24 +9906,24 @@
       <c r="A71" s="18" t="n">
         <v>46309</v>
       </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B71" s="19" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>D15b</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
+          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d15b-color-p2</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -9938,17 +9938,17 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
+          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 3a41eb7</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
     </row>
@@ -9958,22 +9958,22 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>开始</t>
+          <t>根因</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D15b</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
+          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 26e69ec soak8h</t>
+          <t>dr1v90 task/d15b-color-p2</t>
         </is>
       </c>
     </row>
@@ -9981,24 +9981,24 @@
       <c r="A74" s="18" t="n">
         <v>46309</v>
       </c>
-      <c r="B74" s="19" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B74" s="14" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
+          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 3a41eb7</t>
         </is>
       </c>
     </row>
@@ -10006,9 +10006,9 @@
       <c r="A75" s="18" t="n">
         <v>46309</v>
       </c>
-      <c r="B75" s="16" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>开始</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
@@ -10018,62 +10018,62 @@
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
+          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 5cbe79f</t>
+          <t>dr1v90 26e69ec soak8h</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="18" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B76" s="14" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B76" s="19" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
+          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 b0f6b5d</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="18" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B77" s="14" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B77" s="16" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
+          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 71d006f / 473abcf</t>
+          <t>dr1v90 5cbe79f</t>
         </is>
       </c>
     </row>
@@ -10088,17 +10088,17 @@
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
+          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 596b191</t>
+          <t>dr1v90 b0f6b5d</t>
         </is>
       </c>
     </row>
@@ -10106,24 +10106,24 @@
       <c r="A79" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B79" s="16" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B79" s="14" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
+          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 60c619a / 596b191</t>
+          <t>dr1v90 71d006f / 473abcf</t>
         </is>
       </c>
     </row>
@@ -10133,7 +10133,7 @@
       </c>
       <c r="B80" s="14" t="inlineStr">
         <is>
-          <t>复验通过</t>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
@@ -10143,12 +10143,12 @@
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
+          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 9bf16ad</t>
+          <t>dr1v90 596b191</t>
         </is>
       </c>
     </row>
@@ -10156,24 +10156,24 @@
       <c r="A81" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B81" s="12" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B81" s="16" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
+          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 60c619a / 596b191</t>
         </is>
       </c>
     </row>
@@ -10188,17 +10188,17 @@
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
+          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 6a373d3</t>
+          <t>dr1v90 9bf16ad</t>
         </is>
       </c>
     </row>
@@ -10206,24 +10206,24 @@
       <c r="A83" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B83" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B83" s="12" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
+          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 cdf49c6</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -10231,24 +10231,24 @@
       <c r="A84" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B84" s="16" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B84" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
+          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 6a373d3</t>
         </is>
       </c>
     </row>
@@ -10256,9 +10256,9 @@
       <c r="A85" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B85" s="16" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B85" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
@@ -10268,12 +10268,12 @@
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
+          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 cdf49c6</t>
         </is>
       </c>
     </row>
@@ -10281,24 +10281,24 @@
       <c r="A86" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B86" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B86" s="16" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
+          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 44ed2cd</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -10306,19 +10306,19 @@
       <c r="A87" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B87" s="12" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B87" s="16" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
+          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
@@ -10338,17 +10338,17 @@
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
+          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ffbfeeb</t>
+          <t>dr1v90 44ed2cd</t>
         </is>
       </c>
     </row>
@@ -10356,19 +10356,19 @@
       <c r="A89" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B89" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B89" s="12" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
+          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
@@ -10381,24 +10381,24 @@
       <c r="A90" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B90" s="12" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B90" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
+          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 ffbfeeb</t>
         </is>
       </c>
     </row>
@@ -10406,24 +10406,24 @@
       <c r="A91" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B91" s="16" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B91" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
+          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 764f81d</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -10438,12 +10438,12 @@
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
+          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
@@ -10456,24 +10456,24 @@
       <c r="A93" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B93" s="20" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B93" s="16" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
+          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d13-boot fdbb217</t>
+          <t>dr1v90 764f81d</t>
         </is>
       </c>
     </row>
@@ -10481,9 +10481,9 @@
       <c r="A94" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B94" s="16" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B94" s="12" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
@@ -10493,7 +10493,7 @@
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
+          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
@@ -10506,24 +10506,24 @@
       <c r="A95" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B95" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B95" s="20" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
+          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 1995be8</t>
+          <t>dr1v90 task/d13-boot fdbb217</t>
         </is>
       </c>
     </row>
@@ -10531,19 +10531,19 @@
       <c r="A96" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B96" s="19" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B96" s="16" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>D3;D4;D5</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
+          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
@@ -10556,20 +10556,24 @@
       <c r="A97" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B97" s="19" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C97" s="7" t="inlineStr"/>
+      <c r="B97" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
+        </is>
+      </c>
+      <c r="C97" s="7" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
+          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>dr1v90 1995be8</t>
         </is>
       </c>
     </row>
@@ -10577,20 +10581,24 @@
       <c r="A98" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B98" s="20" t="inlineStr">
-        <is>
-          <t>里程碑</t>
-        </is>
-      </c>
-      <c r="C98" s="7" t="inlineStr"/>
+      <c r="B98" s="19" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>D3;D4;D5</t>
+        </is>
+      </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
+          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -10606,12 +10614,12 @@
       <c r="C99" s="7" t="inlineStr"/>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
+          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_arch_common_front_display_backend.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -10619,24 +10627,20 @@
       <c r="A100" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B100" s="19" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C100" s="7" t="inlineStr">
-        <is>
-          <t>D3</t>
-        </is>
-      </c>
+      <c r="B100" s="20" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="inlineStr"/>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
+          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
         </is>
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -10649,19 +10653,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C101" s="7" t="inlineStr">
-        <is>
-          <t>D11</t>
-        </is>
-      </c>
+      <c r="C101" s="7" t="inlineStr"/>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
+          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_arch_common_front_display_backend.md</t>
         </is>
       </c>
     </row>
@@ -10676,12 +10676,12 @@
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>D12;D13;D14</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
+          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
         </is>
       </c>
       <c r="E102" s="7" t="inlineStr">
@@ -10701,12 +10701,12 @@
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
@@ -10726,12 +10726,12 @@
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>D15;D16</t>
+          <t>D12;D13;D14</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
@@ -10751,17 +10751,17 @@
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>KR5.2</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 49031f6</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -10769,19 +10769,19 @@
       <c r="A106" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B106" s="16" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B106" s="19" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D15;D16</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
@@ -10794,18 +10794,68 @@
       <c r="A107" s="18" t="n">
         <v>46308</v>
       </c>
-      <c r="B107" s="20" t="inlineStr">
+      <c r="B107" s="19" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C107" s="7" t="inlineStr">
+        <is>
+          <t>KR5.2</t>
+        </is>
+      </c>
+      <c r="D107" s="7" t="inlineStr">
+        <is>
+          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+        </is>
+      </c>
+      <c r="E107" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 49031f6</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="18" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B108" s="16" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C108" s="7" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="D108" s="7" t="inlineStr">
+        <is>
+          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+        </is>
+      </c>
+      <c r="E108" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="18" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B109" s="20" t="inlineStr">
         <is>
           <t>里程碑</t>
         </is>
       </c>
-      <c r="C107" s="7" t="inlineStr"/>
-      <c r="D107" s="7" t="inlineStr">
+      <c r="C109" s="7" t="inlineStr"/>
+      <c r="D109" s="7" t="inlineStr">
         <is>
           <t>显性目的进度看板第一版建立：10 个显性目的 + KR 趋势 + 燃起图 + 里程碑趋势</t>
         </is>
       </c>
-      <c r="E107" s="7" t="inlineStr">
+      <c r="E109" s="7" t="inlineStr">
         <is>
           <t>claude_memory/project_progress_dashboard.md</t>
         </is>

</xml_diff>

<commit_message>
[进度] 10-15 15:05 重新生成
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-15.xlsx
+++ b/docs/progress/显性目的进度_2026-10-15.xlsx
@@ -8528,7 +8528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J121"/>
+  <dimension ref="A1:J123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10098,51 +10098,51 @@
     </row>
     <row r="68">
       <c r="A68" s="20" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B68" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46310</v>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>上行出口全量复验 45/0, 合主线</t>
+          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 fdb4de6</t>
+          <t>dr1v90 task/d21-nband adeba44</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="20" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B69" s="12" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+        <v>46310</v>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D20/D22</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
+          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>scratchpad/v_pls4_board.log</t>
+          <t>~/realspin/tcp</t>
         </is>
       </c>
     </row>
@@ -10150,24 +10150,24 @@
       <c r="A70" s="20" t="n">
         <v>46309</v>
       </c>
-      <c r="B70" s="18" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
+          <t>上行出口全量复验 45/0, 合主线</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>dr1v90 fdb4de6</t>
         </is>
       </c>
     </row>
@@ -10175,24 +10175,24 @@
       <c r="A71" s="20" t="n">
         <v>46309</v>
       </c>
-      <c r="B71" s="18" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
+          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>scratchpad/v_pls4_board.log</t>
         </is>
       </c>
     </row>
@@ -10200,24 +10200,24 @@
       <c r="A72" s="20" t="n">
         <v>46309</v>
       </c>
-      <c r="B72" s="21" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B72" s="18" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
+          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>project_short_term_delivery_1013</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -10232,17 +10232,17 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
+          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 debd3cd</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -10250,24 +10250,24 @@
       <c r="A74" s="20" t="n">
         <v>46309</v>
       </c>
-      <c r="B74" s="12" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B74" s="21" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
+          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>scratchpad v_pls6_board.log</t>
+          <t>project_short_term_delivery_1013</t>
         </is>
       </c>
     </row>
@@ -10275,9 +10275,9 @@
       <c r="A75" s="20" t="n">
         <v>46309</v>
       </c>
-      <c r="B75" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B75" s="18" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
@@ -10287,12 +10287,12 @@
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
+          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>dr1v90 task/pls-2047 debd3cd</t>
         </is>
       </c>
     </row>
@@ -10300,24 +10300,24 @@
       <c r="A76" s="20" t="n">
         <v>46309</v>
       </c>
-      <c r="B76" s="18" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B76" s="12" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
+          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16-ddr 539d303</t>
+          <t>scratchpad v_pls6_board.log</t>
         </is>
       </c>
     </row>
@@ -10325,24 +10325,24 @@
       <c r="A77" s="20" t="n">
         <v>46309</v>
       </c>
-      <c r="B77" s="21" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B77" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
+          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>feedback_save_weekly_quota</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -10350,24 +10350,24 @@
       <c r="A78" s="20" t="n">
         <v>46309</v>
       </c>
-      <c r="B78" s="16" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B78" s="18" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
+          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>dr1v90 task/d16-ddr 539d303</t>
         </is>
       </c>
     </row>
@@ -10375,24 +10375,24 @@
       <c r="A79" s="20" t="n">
         <v>46309</v>
       </c>
-      <c r="B79" s="14" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B79" s="21" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
+          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 2364e5c</t>
+          <t>feedback_save_weekly_quota</t>
         </is>
       </c>
     </row>
@@ -10407,17 +10407,17 @@
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
+          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>用户在场实转</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -10425,24 +10425,24 @@
       <c r="A81" s="20" t="n">
         <v>46309</v>
       </c>
-      <c r="B81" s="21" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B81" s="14" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
+          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 2364e5c</t>
         </is>
       </c>
     </row>
@@ -10450,24 +10450,24 @@
       <c r="A82" s="20" t="n">
         <v>46309</v>
       </c>
-      <c r="B82" s="14" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B82" s="16" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
+          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>用户在场实转</t>
         </is>
       </c>
     </row>
@@ -10482,12 +10482,12 @@
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
+          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
@@ -10507,17 +10507,17 @@
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
+          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 dee9be6</t>
+          <t>dr1v90 task/d18-pl-default d35c6d4</t>
         </is>
       </c>
     </row>
@@ -10525,24 +10525,24 @@
       <c r="A85" s="20" t="n">
         <v>46309</v>
       </c>
-      <c r="B85" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B85" s="21" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>D15b</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
+          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d15b-color-p2</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -10557,17 +10557,17 @@
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
+          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 3a41eb7</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
     </row>
@@ -10577,22 +10577,22 @@
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>开始</t>
+          <t>根因</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D15b</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
+          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 26e69ec soak8h</t>
+          <t>dr1v90 task/d15b-color-p2</t>
         </is>
       </c>
     </row>
@@ -10600,24 +10600,24 @@
       <c r="A88" s="20" t="n">
         <v>46309</v>
       </c>
-      <c r="B88" s="21" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
+          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 3a41eb7</t>
         </is>
       </c>
     </row>
@@ -10625,9 +10625,9 @@
       <c r="A89" s="20" t="n">
         <v>46309</v>
       </c>
-      <c r="B89" s="18" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B89" s="6" t="inlineStr">
+        <is>
+          <t>开始</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
@@ -10637,62 +10637,62 @@
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
+          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 5cbe79f</t>
+          <t>dr1v90 26e69ec soak8h</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="20" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B90" s="14" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B90" s="21" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
+          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 b0f6b5d</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="20" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B91" s="14" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B91" s="18" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
+          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 71d006f / 473abcf</t>
+          <t>dr1v90 5cbe79f</t>
         </is>
       </c>
     </row>
@@ -10707,17 +10707,17 @@
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
+          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 596b191</t>
+          <t>dr1v90 b0f6b5d</t>
         </is>
       </c>
     </row>
@@ -10725,24 +10725,24 @@
       <c r="A93" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B93" s="18" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B93" s="14" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
+          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 60c619a / 596b191</t>
+          <t>dr1v90 71d006f / 473abcf</t>
         </is>
       </c>
     </row>
@@ -10752,7 +10752,7 @@
       </c>
       <c r="B94" s="14" t="inlineStr">
         <is>
-          <t>复验通过</t>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
@@ -10762,12 +10762,12 @@
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
+          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 9bf16ad</t>
+          <t>dr1v90 596b191</t>
         </is>
       </c>
     </row>
@@ -10775,24 +10775,24 @@
       <c r="A95" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B95" s="12" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B95" s="18" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
+          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 60c619a / 596b191</t>
         </is>
       </c>
     </row>
@@ -10807,17 +10807,17 @@
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
+          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 6a373d3</t>
+          <t>dr1v90 9bf16ad</t>
         </is>
       </c>
     </row>
@@ -10825,24 +10825,24 @@
       <c r="A97" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B97" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B97" s="12" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
+          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 cdf49c6</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -10850,24 +10850,24 @@
       <c r="A98" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B98" s="18" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B98" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
+          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 6a373d3</t>
         </is>
       </c>
     </row>
@@ -10875,9 +10875,9 @@
       <c r="A99" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B99" s="18" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B99" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
@@ -10887,12 +10887,12 @@
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
+          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 cdf49c6</t>
         </is>
       </c>
     </row>
@@ -10900,24 +10900,24 @@
       <c r="A100" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B100" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B100" s="18" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
+          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
         </is>
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 44ed2cd</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -10925,19 +10925,19 @@
       <c r="A101" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B101" s="12" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B101" s="18" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
+          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
@@ -10957,17 +10957,17 @@
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
+          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
         </is>
       </c>
       <c r="E102" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ffbfeeb</t>
+          <t>dr1v90 44ed2cd</t>
         </is>
       </c>
     </row>
@@ -10975,19 +10975,19 @@
       <c r="A103" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B103" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B103" s="12" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
+          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
@@ -11000,24 +11000,24 @@
       <c r="A104" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B104" s="12" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B104" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
+          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 ffbfeeb</t>
         </is>
       </c>
     </row>
@@ -11025,24 +11025,24 @@
       <c r="A105" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B105" s="18" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B105" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
+          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 764f81d</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -11057,12 +11057,12 @@
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
+          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
@@ -11075,24 +11075,24 @@
       <c r="A107" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B107" s="16" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B107" s="18" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
+          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d13-boot fdbb217</t>
+          <t>dr1v90 764f81d</t>
         </is>
       </c>
     </row>
@@ -11100,9 +11100,9 @@
       <c r="A108" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B108" s="18" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B108" s="12" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
@@ -11112,7 +11112,7 @@
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
+          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
@@ -11125,24 +11125,24 @@
       <c r="A109" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B109" s="14" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B109" s="16" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
+          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 1995be8</t>
+          <t>dr1v90 task/d13-boot fdbb217</t>
         </is>
       </c>
     </row>
@@ -11150,19 +11150,19 @@
       <c r="A110" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B110" s="21" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B110" s="18" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>D3;D4;D5</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
+          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
         </is>
       </c>
       <c r="E110" s="7" t="inlineStr">
@@ -11175,20 +11175,24 @@
       <c r="A111" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B111" s="21" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C111" s="7" t="inlineStr"/>
+      <c r="B111" s="14" t="inlineStr">
+        <is>
+          <t>复验通过</t>
+        </is>
+      </c>
+      <c r="C111" s="7" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
+          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>dr1v90 1995be8</t>
         </is>
       </c>
     </row>
@@ -11196,20 +11200,24 @@
       <c r="A112" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B112" s="16" t="inlineStr">
-        <is>
-          <t>里程碑</t>
-        </is>
-      </c>
-      <c r="C112" s="7" t="inlineStr"/>
+      <c r="B112" s="21" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C112" s="7" t="inlineStr">
+        <is>
+          <t>D3;D4;D5</t>
+        </is>
+      </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
+          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
         </is>
       </c>
       <c r="E112" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -11225,12 +11233,12 @@
       <c r="C113" s="7" t="inlineStr"/>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
+          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_arch_common_front_display_backend.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -11238,24 +11246,20 @@
       <c r="A114" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B114" s="21" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C114" s="7" t="inlineStr">
-        <is>
-          <t>D3</t>
-        </is>
-      </c>
+      <c r="B114" s="16" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="C114" s="7" t="inlineStr"/>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
+          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -11268,19 +11272,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C115" s="7" t="inlineStr">
-        <is>
-          <t>D11</t>
-        </is>
-      </c>
+      <c r="C115" s="7" t="inlineStr"/>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
+          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_arch_common_front_display_backend.md</t>
         </is>
       </c>
     </row>
@@ -11295,12 +11295,12 @@
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>D12;D13;D14</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
+          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
         </is>
       </c>
       <c r="E116" s="7" t="inlineStr">
@@ -11320,12 +11320,12 @@
       </c>
       <c r="C117" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
@@ -11345,12 +11345,12 @@
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>D15;D16</t>
+          <t>D12;D13;D14</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
         </is>
       </c>
       <c r="E118" s="7" t="inlineStr">
@@ -11370,17 +11370,17 @@
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>KR5.2</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 49031f6</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -11388,19 +11388,19 @@
       <c r="A120" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B120" s="18" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B120" s="21" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D15;D16</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
         </is>
       </c>
       <c r="E120" s="7" t="inlineStr">
@@ -11413,18 +11413,68 @@
       <c r="A121" s="20" t="n">
         <v>46308</v>
       </c>
-      <c r="B121" s="16" t="inlineStr">
+      <c r="B121" s="21" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t>KR5.2</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 49031f6</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="20" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B122" s="18" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C122" s="7" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="D122" s="7" t="inlineStr">
+        <is>
+          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+        </is>
+      </c>
+      <c r="E122" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="20" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B123" s="16" t="inlineStr">
         <is>
           <t>里程碑</t>
         </is>
       </c>
-      <c r="C121" s="7" t="inlineStr"/>
-      <c r="D121" s="7" t="inlineStr">
+      <c r="C123" s="7" t="inlineStr"/>
+      <c r="D123" s="7" t="inlineStr">
         <is>
           <t>显性目的进度看板第一版建立：10 个显性目的 + KR 趋势 + 燃起图 + 里程碑趋势</t>
         </is>
       </c>
-      <c r="E121" s="7" t="inlineStr">
+      <c r="E123" s="7" t="inlineStr">
         <is>
           <t>claude_memory/project_progress_dashboard.md</t>
         </is>

</xml_diff>